<commit_message>
Inventory import: default duplicates to Skip existing, show parsed dates in preview, template uses UK dd/mm/yyyy
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/Inventory_Import_Template.xlsx
+++ b/public/templates/Inventory_Import_Template.xlsx
@@ -308,7 +308,7 @@
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Expiry of the stock batch (stock row only).
-Format: YYYY-MM-DD, e.g. 2027-12-31. Do NOT type 31/12/2027: text dates are read as US month/day.</t>
+Format: UK date dd/mm/yyyy, e.g. 31/12/2027 (also dd-mm-yyyy, dd.mm.yyyy, YYYY-MM-DD or a real Excel date). mm/yyyy means the last day of that month. Impossible dates (31/02/2027) are left blank with a warning.</t>
       </text>
     </comment>
     <comment ref="W1" authorId="0" shapeId="0">
@@ -320,7 +320,7 @@
     <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <t>Optional. Informational. Read by the importer but not currently saved on the product.
-Format: YYYY-MM-DD.</t>
+Format: UK date dd/mm/yyyy, e.g. 13/10/2026.</t>
       </text>
     </comment>
     <comment ref="Y1" authorId="0" shapeId="0">
@@ -873,7 +873,7 @@
       </c>
       <c r="V2" s="3" t="inlineStr">
         <is>
-          <t>2027-12-31</t>
+          <t>31/12/2027</t>
         </is>
       </c>
       <c r="W2" s="4" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="X2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="Y2" s="4" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="V3" s="3" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>30/06/2028</t>
         </is>
       </c>
       <c r="W3" s="4" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="Y3" s="4" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="Y4" s="4" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="V5" s="3" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>31/03/2027</t>
         </is>
       </c>
       <c r="W5" s="4" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="Y5" s="4" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="Y6" s="4" t="inlineStr">
@@ -11294,7 +11294,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5. "Duplicate SKUs": Update existing overwrites products with the same SKU; Skip existing leaves them untouched.</t>
+          <t>5. "Duplicate SKUs": Skip existing (the default) leaves products with the same SKU untouched; Update existing overwrites them.</t>
         </is>
       </c>
     </row>
@@ -11315,7 +11315,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8. Dates: use YYYY-MM-DD (e.g. 2027-12-31) or real Excel date cells. Text such as 31/12/2027 is read as month/day and goes wrong.</t>
+          <t>8. Dates are UK day/month/year: dd/mm/yyyy (e.g. 07/10/2026 = 7 October 2026). dd-mm-yyyy, dd.mm.yyyy, 2-digit years (07/10/26), YYYY-MM-DD and real Excel date cells also work. Impossible dates such as 31/02/2026 are left blank and listed as a warning in Preview.</t>
         </is>
       </c>
     </row>
@@ -11934,12 +11934,12 @@
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD, e.g. 2027-12-31. Do NOT type 31/12/2027: text dates are read as US month/day.</t>
+          <t>UK date dd/mm/yyyy, e.g. 31/12/2027 (also dd-mm-yyyy, dd.mm.yyyy, YYYY-MM-DD or a real Excel date). mm/yyyy means the last day of that month. Impossible dates (31/02/2027) are left blank with a warning.</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>2027-12-31</t>
+          <t>31/12/2027</t>
         </is>
       </c>
     </row>
@@ -11988,12 +11988,12 @@
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD.</t>
+          <t>UK date dd/mm/yyyy, e.g. 13/10/2026.</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>13/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>